<commit_message>
fix(resolver_runtime): promote command centre plug and play notion defaults [Mandor-Gate: PASSED | Sandbox-Override: Executed manually]
</commit_message>
<xml_diff>
--- a/BOSMAX_AVATAR_CONTEXT_RESOLVER_v1.xlsx
+++ b/BOSMAX_AVATAR_CONTEXT_RESOLVER_v1.xlsx
@@ -12,9 +12,11 @@
     <sheet name="MANNEQUIN_POSE_LIBRARY" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="SCENE_CONTEXT_LIBRARY" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="ROTATION_POOLS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="NOTION_EXPORT_VIEW" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="VALIDATION_RULES" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="CHANGELOG" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CC_AVATAR_ID_VIEW" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CC_AVATAR_POOL_VIEW" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="NOTION_EXPORT_VIEW" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="VALIDATION_RULES" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="CHANGELOG" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1302,6 +1304,48 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Timestamp_UTC</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Change_Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-06-05T14:30:34+00:00</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Generated first-pass avatar context resolver and rotation pool for stealth male batch prompting with Command Centre beginner selector views.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2491,130 +2535,118 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Rule_ID</t>
+          <t>Pool_ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Rule_Description</t>
+          <t>Display_Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Product_ID</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Product_Family</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Silo</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Rotation_Mode</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>No_Repeat_Window</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Minimum_Approved_Count</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Safe_Usage_Notes</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AVATAR_CONTEXT_ID_NOT_FOUND</t>
+          <t>BOSMAX_MALE_STEALTH_POOL_001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Fail closed if Avatar_Context_ID cannot resolve from the runtime registry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AVATAR_POOL_ID_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Fail closed if Avatar_Pool_ID cannot resolve from the runtime registry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>AVATAR_STATUS_INVALID</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fail closed if Runtime_Allowed is true but Status is not APPROVED, LOCKED, or SEED_READY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>AVATAR_SILO_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Fail closed if template silo is not included in Silo_Allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AVATAR_PRODUCT_FAMILY_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Fail closed if product family is not included in Product_Family_Allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AVATAR_CAMERA_STYLE_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Fail closed if camera style is not included in Camera_Style_Allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AVATAR_PHYSICS_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Fail closed if mannequin pose is incompatible with requested Physics class.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>AVATAR_POOL_REPEAT_WINDOW</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Fail closed if AUTO_ROTATE cannot satisfy the configured no-repeat window.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>UNSAFE_MANUAL_OVERRIDE</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Fail closed if manual override is present without Needs Compliance Review.</t>
+          <t>BOSMAX Male Stealth Pool | BOSMAX Serum Family</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>BOSMAX_SERUM</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ROUND_ROBIN_NO_REPEAT</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>7</v>
+      </c>
+      <c r="H2" t="n">
+        <v>8</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Repo-owned AUTO_ROTATE pool for BOSMAX Serum stealth batch runs. Notion may display IDs only; manual override requires Needs Compliance Review.</t>
         </is>
       </c>
     </row>
@@ -2629,34 +2661,728 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="31" customWidth="1" min="7" max="7"/>
+    <col width="32" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Avatar_Context_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Display_Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Persona_Label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Gender</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Age_Range</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Silo_Allowed</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Product_Family_Allowed</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Scene_Label</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Mannequin_Label</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Camera_Style_Allowed</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Safe_Usage_Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>RIZAL | RIZAL_CASUAL_01 | Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>27-34</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Close Hold Reset</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona RIZAL with RIZAL_CASUAL_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>RIZAL | RIZAL_ACTIVE_01 | Morning Street Confidence Walk</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>27-34</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Morning Street Confidence Walk</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Walk And Talk</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona RIZAL with RIZAL_ACTIVE_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>RIZAL | RIZAL_SMART_01 | Office Confidence Corner</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>27-34</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Office Confidence Corner</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Desk Reveal Confidence</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona RIZAL with RIZAL_SMART_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>RIZAL | RIZAL_RAYA_01 | Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>27-34</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Close Hold Reset</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona RIZAL with RIZAL_RAYA_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>AZMAN | AZMAN_CASUAL_01 | Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Azman</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Close Hold Reset</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona AZMAN with AZMAN_CASUAL_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>AZMAN | AZMAN_SMART_01 | Office Confidence Corner</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Azman</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Office Confidence Corner</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Desk Reveal Confidence</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona AZMAN with AZMAN_SMART_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>AZMAN | AZMAN_ACTIVE_01 | Morning Street Confidence Walk</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Azman</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Morning Street Confidence Walk</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Walk And Talk</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona AZMAN with AZMAN_ACTIVE_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>BOSMAX_AVP_0008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AZMAN | AZMAN_RAYA_01 | Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Azman</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>FAMILY_MALE_EXT_SENSITIVE_OIL</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Close Hold Reset</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>STEALTH resolver pack for BOSMAX Serum family. Persona AZMAN with AZMAN_RAYA_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Timestamp_UTC</t>
+          <t>Rule_ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Change_Note</t>
+          <t>Rule_Description</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-05T13:55:09+00:00</t>
+          <t>AVATAR_CONTEXT_ID_NOT_FOUND</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Generated first-pass avatar context resolver and rotation pool for stealth male batch prompting.</t>
+          <t>Fail closed if Avatar_Context_ID cannot resolve from the runtime registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AVATAR_POOL_ID_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fail closed if Avatar_Pool_ID cannot resolve from the runtime registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AVATAR_STATUS_INVALID</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fail closed if Runtime_Allowed is true but Status is not APPROVED, LOCKED, or SEED_READY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AVATAR_SILO_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fail closed if template silo is not included in Silo_Allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AVATAR_PRODUCT_FAMILY_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fail closed if product family is not included in Product_Family_Allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AVATAR_CAMERA_STYLE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fail closed if camera style is not included in Camera_Style_Allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AVATAR_PHYSICS_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fail closed if mannequin pose is incompatible with requested Physics class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AVATAR_POOL_REPEAT_WINDOW</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fail closed if AUTO_ROTATE cannot satisfy the configured no-repeat window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>UNSAFE_MANUAL_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fail closed if manual override is present without Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>COMMAND_CENTRE_AVATAR_VIEW_ONLY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Command Centre avatar and pool views must remain frontend-safe selector surfaces only.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(resolver_runtime): add command centre product workflows for stealth direct and session-only [Mandor-Gate: PASSED | Sandbox-Override: Executed manually]
</commit_message>
<xml_diff>
--- a/BOSMAX_AVATAR_CONTEXT_RESOLVER_v1.xlsx
+++ b/BOSMAX_AVATAR_CONTEXT_RESOLVER_v1.xlsx
@@ -9,14 +9,15 @@
   <sheets>
     <sheet name="AVATAR_CONTEXT_PACKS" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="AVATAR_PERSONA_INDEX" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MANNEQUIN_POSE_LIBRARY" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="SCENE_CONTEXT_LIBRARY" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ROTATION_POOLS" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CC_AVATAR_ID_VIEW" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CC_AVATAR_POOL_VIEW" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="NOTION_EXPORT_VIEW" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="VALIDATION_RULES" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="CHANGELOG" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="VIEW_ALIASES" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="MANNEQUIN_POSE_LIBRARY" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="SCENE_CONTEXT_LIBRARY" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ROTATION_POOLS" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CC_AVATAR_ID_VIEW" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CC_AVATAR_POOL_VIEW" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="NOTION_EXPORT_VIEW" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="VALIDATION_RULES" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="CHANGELOG" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,10 +435,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S9"/>
+  <dimension ref="A1:S11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
@@ -1299,12 +1300,360 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MWCB_DIRECT_AVP_0001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RIZAL | RIZAL_CASUAL_01 | Household Relief Shelf Reset</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>RIZAL</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>MALAY_MALE_YOUNG_01</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>27-34</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>CTX_HOME_TRAD_REMEDY_001</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>MAN_DIRECT_BOTTLE_PICKUP_001</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>RIZAL_CASUAL_01</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>avatars/RIZAL.yaml::prompt_fragment</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="P10" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>DIRECT resolver pack for Minyak Warisan Cap Burung family. Persona RIZAL with RIZAL_CASUAL_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Wardrobe sourced from RIZAL.yaml::RIZAL_CASUAL_01; scene keyed from mwcb_home_relief; mannequin pose resolved in avatar context builder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MWCB_DIRECT_AVP_0002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AZMAN | AZMAN_CASUAL_01 | On-The-Go Remedy Grab</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>AZMAN</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>MALAY_MALE_YOUNG_01</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>CTX_TRAVEL_TRAD_REMEDY_001</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>MAN_DIRECT_BAG_REACH_001</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>AZMAN_CASUAL_01</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>NONE</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>avatars/AZMAN.yaml::prompt_fragment</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="P11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>DIRECT resolver pack for Minyak Warisan Cap Burung family. Persona AZMAN with AZMAN_CASUAL_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Wardrobe sourced from AZMAN.yaml::AZMAN_CASUAL_01; scene keyed from mwcb_bag_ready; mannequin pose resolved in avatar context builder.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Rule_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Rule_Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AVATAR_CONTEXT_ID_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fail closed if Avatar_Context_ID cannot resolve from the runtime registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AVATAR_POOL_ID_NOT_FOUND</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Fail closed if Avatar_Pool_ID cannot resolve from the runtime registry.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AVATAR_STATUS_INVALID</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fail closed if Runtime_Allowed is true but Status is not APPROVED, LOCKED, or SEED_READY.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AVATAR_SILO_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Fail closed if template silo is not included in Silo_Allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AVATAR_PRODUCT_FAMILY_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Fail closed if product family is not included in Product_Family_Allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AVATAR_CAMERA_STYLE_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Fail closed if camera style is not included in Camera_Style_Allowed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AVATAR_PHYSICS_MISMATCH</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Fail closed if mannequin pose is incompatible with requested Physics class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>AVATAR_POOL_REPEAT_WINDOW</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Fail closed if AUTO_ROTATE cannot satisfy the configured no-repeat window.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>UNSAFE_MANUAL_OVERRIDE</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Fail closed if manual override is present without Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>COMMAND_CENTRE_AVATAR_VIEW_ONLY</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Command Centre avatar and pool views must remain frontend-safe selector surfaces only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>COMMAND_CENTRE_PRODUCT_WORKFLOW_SUPPORT</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Registered Command Centre workflows must expose separate STEALTH and DIRECT avatar support without leaking prompt internals.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1332,12 +1681,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-05T14:30:34+00:00</t>
+          <t>2026-06-05T15:02:33+00:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Generated first-pass avatar context resolver and rotation pool for stealth male batch prompting with Command Centre beginner selector views.</t>
+          <t>Generated avatar context resolver and rotation pools for BOSMAX STEALTH and MWCB DIRECT Command Centre workflows with workbook aliases and beginner selector views.</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1707,7 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="31" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="37" customWidth="1" min="7" max="7"/>
@@ -1419,7 +1768,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>BOSMAX_SERUM | MAVERIX_MAXOIL</t>
+          <t>BOSMAX_SERUM | CAP_BURUNG_MINYAK | MAVERIX_MAXOIL</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1454,7 +1803,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>BOSMAX_SERUM | MAVERIX_MAXOIL</t>
+          <t>BOSMAX_SERUM | CAP_BURUNG_MINYAK | MAVERIX_MAXOIL</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1482,7 +1831,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Public_View_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Workbook_Sheet_Alias</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>NOTION_COMMAND_CENTRE_AVATAR_ID_VIEW</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>CC_AVATAR_ID_VIEW</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Generic beginner avatar selector view across approved runtime packs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NOTION_COMMAND_CENTRE_AVATAR_POOL_VIEW</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CC_AVATAR_POOL_VIEW</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Generic beginner avatar pool selector view across approved runtime pools.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -1621,174 +2040,67 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Scene_Context_ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Scene_Label</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Base_Scene_Key</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Environment_Summary</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Silo_Allowed</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Camera_Style_Allowed</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Safe_Usage_Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>CTX_HOME_STEALTH_RESET_001</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Quiet Home Reset Corner</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>home_indoor</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Warm indoor private corner with low-noise everyday props and product-neutral framing.</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>STEALTH</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>MAN_DIRECT_BOTTLE_PICKUP_001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Bottle Pickup Utility</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Natural household reach, bottle pickup, or side-table explanation gesture with grounded family-man practicality.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CLASS_A</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
         <is>
           <t>UGC_IPHONE_RAW</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Private indoor stealth lane. Keep framing conversational and product-neutral.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>CTX_STREET_MORNING_RESET_001</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Morning Street Confidence Walk</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>outdoor_street</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Soft daylight outdoor walkway with authentic motion and subtle background depth.</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>STEALTH</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>CTX_HOME_TRAD_REMEDY_001</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MAN_DIRECT_BAG_REACH_001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Bag Reach Practicality</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Simple bag, drawer, or car-pocket reach motion showing compact everyday-carry readiness without exaggerated acting.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>CLASS_A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>UGC_IPHONE_RAW</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Outdoor stealth lane. Keep gestures natural and avoid fitness-bro exaggeration.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CTX_OFFICE_CONFIDENCE_CORNER_001</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Office Confidence Corner</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>office_interior</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Smart indoor office nook with grounded professional texture and light desk cues.</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>STEALTH</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>UGC_IPHONE_RAW</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Professional stealth lane. Keep the setting calm and non-clinical.</t>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>CTX_TRAVEL_TRAD_REMEDY_001</t>
         </is>
       </c>
     </row>
@@ -1803,12 +2115,257 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:G6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Scene_Context_ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Scene_Label</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Base_Scene_Key</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Environment_Summary</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Silo_Allowed</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Camera_Style_Allowed</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Safe_Usage_Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CTX_HOME_STEALTH_RESET_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Quiet Home Reset Corner</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>home_indoor</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Warm indoor private corner with low-noise everyday props and product-neutral framing.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Private indoor stealth lane. Keep framing conversational and product-neutral.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>CTX_STREET_MORNING_RESET_001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Morning Street Confidence Walk</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>outdoor_street</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Soft daylight outdoor walkway with authentic motion and subtle background depth.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Outdoor stealth lane. Keep gestures natural and avoid fitness-bro exaggeration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CTX_OFFICE_CONFIDENCE_CORNER_001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Office Confidence Corner</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>office_interior</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Smart indoor office nook with grounded professional texture and light desk cues.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>STEALTH</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Professional stealth lane. Keep the setting calm and non-clinical.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>CTX_HOME_TRAD_REMEDY_001</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Household Relief Shelf Reset</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>mwcb_home_relief</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Warm rumah setting with small household storage cues, everyday reachability, and practical family utility framing.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>DIRECT traditional-remedy lane. Keep the bottle within normal household use context and avoid clinical implication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>CTX_TRAVEL_TRAD_REMEDY_001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>On-The-Go Remedy Grab</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>mwcb_bag_ready</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Natural grab-from-bag or dashboard-side readiness moment showing compact everyday carry practicality.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>DIRECT traditional-remedy lane. Keep usage practical, pocketable, and non-medical.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
@@ -1938,21 +2495,77 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MWCB_TRAD_REMEDY_POOL_001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MWCB Direct Remedy Pool | Minyak Warisan Cap Burung</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CAP_BURUNG_MINYAK</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>MWCB_DIRECT_AVP_0001 | MWCB_DIRECT_AVP_0002</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>ROUND_ROBIN_NO_REPEAT</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="K3" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Repo-owned AUTO_ROTATE pool for Minyak Warisan Cap Burung DIRECT batch runs. Notion may display IDs only; manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -2524,23 +3137,147 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MWCB_DIRECT_AVP_0001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>RIZAL | RIZAL_CASUAL_01 | Household Relief Shelf Reset</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>27-34</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Household Relief Shelf Reset</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Bottle Pickup Utility</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>DIRECT resolver pack for Minyak Warisan Cap Burung family. Persona RIZAL with RIZAL_CASUAL_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MWCB_DIRECT_AVP_0002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>AZMAN | AZMAN_CASUAL_01 | On-The-Go Remedy Grab</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Azman</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>On-The-Go Remedy Grab</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Bag Reach Practicality</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>DIRECT resolver pack for Minyak Warisan Cap Burung family. Persona AZMAN with AZMAN_CASUAL_01. Manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
     <col width="31" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
@@ -2650,21 +3387,69 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MWCB_TRAD_REMEDY_POOL_001</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MWCB Direct Remedy Pool | Minyak Warisan Cap Burung</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>CAP_BURUNG_MINYAK</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ROUND_ROBIN_NO_REPEAT</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Repo-owned AUTO_ROTATE pool for Minyak Warisan Cap Burung DIRECT batch runs. Notion may display IDs only; manual override requires Needs Compliance Review.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
@@ -3236,153 +4021,127 @@
         </is>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Rule_ID</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Rule_Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>AVATAR_CONTEXT_ID_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Fail closed if Avatar_Context_ID cannot resolve from the runtime registry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AVATAR_POOL_ID_NOT_FOUND</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Fail closed if Avatar_Pool_ID cannot resolve from the runtime registry.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>AVATAR_STATUS_INVALID</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Fail closed if Runtime_Allowed is true but Status is not APPROVED, LOCKED, or SEED_READY.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>AVATAR_SILO_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Fail closed if template silo is not included in Silo_Allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AVATAR_PRODUCT_FAMILY_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Fail closed if product family is not included in Product_Family_Allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AVATAR_CAMERA_STYLE_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Fail closed if camera style is not included in Camera_Style_Allowed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AVATAR_PHYSICS_MISMATCH</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Fail closed if mannequin pose is incompatible with requested Physics class.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>AVATAR_POOL_REPEAT_WINDOW</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Fail closed if AUTO_ROTATE cannot satisfy the configured no-repeat window.</t>
-        </is>
-      </c>
-    </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>UNSAFE_MANUAL_OVERRIDE</t>
+          <t>MWCB_DIRECT_AVP_0001</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Fail closed if manual override is present without Needs Compliance Review.</t>
+          <t>RIZAL | RIZAL_CASUAL_01 | Household Relief Shelf Reset</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Rizal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>27-34</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Household Relief Shelf Reset</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Bottle Pickup Utility</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>DIRECT resolver pack for Minyak Warisan Cap Burung family. Persona RIZAL with RIZAL_CASUAL_01. Manual override requires Needs Compliance Review.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>COMMAND_CENTRE_AVATAR_VIEW_ONLY</t>
+          <t>MWCB_DIRECT_AVP_0002</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Command Centre avatar and pool views must remain frontend-safe selector surfaces only.</t>
+          <t>AZMAN | AZMAN_CASUAL_01 | On-The-Go Remedy Grab</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Azman</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>30-38</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>FAMILY_TRADITIONAL_REMEDY_OIL</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>On-The-Go Remedy Grab</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Bag Reach Practicality</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>UGC_IPHONE_RAW</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>DIRECT resolver pack for Minyak Warisan Cap Burung family. Persona AZMAN with AZMAN_CASUAL_01. Manual override requires Needs Compliance Review.</t>
         </is>
       </c>
     </row>

</xml_diff>